<commit_message>
remove sdtm_mapping from crf specs
</commit_message>
<xml_diff>
--- a/curation/draft/crf/CRF_QRS_6MWT.xlsx
+++ b/curation/draft/crf/CRF_QRS_6MWT.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_github\cdisc-org\COSMoS\curation\draft\crf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45E182B5-9068-4D00-9711-E1751C885510}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7C3514B-B1E5-4242-B1F7-15601142F4F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CRF_QRS_6MWT!$L$1:$L$1487</definedName>
   </definedNames>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -398,35 +398,6 @@
     <t>FTREASND when FTSTAT=NOT DONE</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">FTORRESU when  FTTESTCD = </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9.5"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Albany AMT"/>
-      </rPr>
-      <t>"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9.5"/>
-        <color rgb="FF000000"/>
-        <rFont val="Albany AMT"/>
-      </rPr>
-      <t>SIXMW101</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9.5"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Albany AMT"/>
-      </rPr>
-      <t>"</t>
-    </r>
-  </si>
-  <si>
     <t>FTORRESU when FTTESTCD = SIXMW102</t>
   </si>
   <si>
@@ -461,6 +432,35 @@
   </si>
   <si>
     <t>2-3</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">FTORRESU when FTTESTCD = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Albany AMT"/>
+      </rPr>
+      <t>"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <color rgb="FF000000"/>
+        <rFont val="Albany AMT"/>
+      </rPr>
+      <t>SIXMW101</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Albany AMT"/>
+      </rPr>
+      <t>"</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -804,7 +804,7 @@
         <v>6</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>7</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>31</v>
@@ -834,7 +834,7 @@
         <v>13</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="S1" s="1" t="s">
         <v>14</v>
@@ -897,20 +897,20 @@
         <v>60</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>33</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F2" s="4"/>
       <c r="G2" s="4" t="s">
         <v>50</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
@@ -983,20 +983,20 @@
         <v>60</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>33</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F3" s="4"/>
       <c r="G3" s="4" t="s">
         <v>50</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
@@ -1059,20 +1059,20 @@
         <v>60</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>33</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="4" t="s">
         <v>50</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
@@ -1087,7 +1087,7 @@
         <v>51</v>
       </c>
       <c r="O4" s="11" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="P4" s="6"/>
       <c r="Q4" s="6" t="s">
@@ -1143,20 +1143,20 @@
         <v>60</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>33</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4" t="s">
         <v>50</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
@@ -1225,7 +1225,7 @@
         <v>33</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F6" s="4"/>
       <c r="G6" s="4" t="s">
@@ -1301,7 +1301,7 @@
         <v>33</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F7" s="4"/>
       <c r="G7" s="4" t="s">
@@ -1366,10 +1366,10 @@
         <v>82</v>
       </c>
       <c r="AH7" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AI7" s="10" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="AJ7" s="6"/>
     </row>
@@ -1385,7 +1385,7 @@
         <v>33</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F8" s="4"/>
       <c r="G8" s="4" t="s">
@@ -1461,7 +1461,7 @@
         <v>33</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F9" s="4"/>
       <c r="G9" s="4" t="s">
@@ -1526,10 +1526,10 @@
         <v>82</v>
       </c>
       <c r="AH9" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AI9" s="10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="AJ9" s="6"/>
     </row>
@@ -1545,7 +1545,7 @@
         <v>33</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="s">
@@ -1621,7 +1621,7 @@
         <v>33</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
@@ -1686,10 +1686,10 @@
         <v>82</v>
       </c>
       <c r="AH11" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AI11" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="AJ11" s="6"/>
     </row>
@@ -1705,7 +1705,7 @@
         <v>33</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F12" s="4"/>
       <c r="G12" s="4" t="s">
@@ -1781,7 +1781,7 @@
         <v>33</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
@@ -1846,10 +1846,10 @@
         <v>82</v>
       </c>
       <c r="AH13" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AI13" s="10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="AJ13" s="6"/>
     </row>
@@ -1865,7 +1865,7 @@
         <v>33</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
@@ -1941,7 +1941,7 @@
         <v>33</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
@@ -2006,10 +2006,10 @@
         <v>82</v>
       </c>
       <c r="AH15" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AI15" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="AJ15" s="6"/>
     </row>
@@ -2025,7 +2025,7 @@
         <v>33</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4" t="s">
@@ -2101,7 +2101,7 @@
         <v>33</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4" t="s">
@@ -2166,10 +2166,10 @@
         <v>82</v>
       </c>
       <c r="AH17" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AI17" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="AJ17" s="6"/>
     </row>

</xml_diff>